<commit_message>
Atualiza Superestrutura · 2026-08-03T15:11:05.828-03:00
Responsável: Júlia
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81044126\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FE54E4D-184F-441A-9C14-8821613DC53F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84B4A7F8-7509-4CEE-955A-803123724AEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2483,7 +2483,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="184">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -2968,6 +2968,8 @@
     <xf numFmtId="0" fontId="30" fillId="24" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3475,7 +3477,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="3">
-        <v>46231</v>
+        <v>46236</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -3511,38 +3513,42 @@
         <v>9</v>
       </c>
       <c r="C15" s="6">
-        <v>69180</v>
+        <v>71300</v>
       </c>
       <c r="D15" s="7"/>
+      <c r="E15" s="184"/>
     </row>
     <row r="16" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="6">
-        <v>57220</v>
+        <v>62700</v>
       </c>
       <c r="D16" s="7"/>
-    </row>
-    <row r="17" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E16" s="184"/>
+    </row>
+    <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="6">
-        <v>56860</v>
+        <v>61240</v>
       </c>
       <c r="D17" s="7"/>
-    </row>
-    <row r="18" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E17" s="185"/>
+    </row>
+    <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C18" s="6">
-        <v>55260</v>
+        <v>56550</v>
       </c>
       <c r="D18" s="7"/>
-    </row>
-    <row r="19" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E18" s="185"/>
+    </row>
+    <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="5" t="s">
         <v>13</v>
       </c>
@@ -3550,17 +3556,19 @@
         <v>30540</v>
       </c>
       <c r="D19" s="7"/>
-    </row>
-    <row r="20" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E19" s="184"/>
+    </row>
+    <row r="20" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="5" t="s">
         <v>14</v>
       </c>
       <c r="C20" s="6">
-        <v>39000</v>
+        <v>44820</v>
       </c>
       <c r="D20" s="7"/>
-    </row>
-    <row r="21" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E20" s="185"/>
+    </row>
+    <row r="21" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
         <v>15</v>
       </c>
@@ -3568,8 +3576,9 @@
         <v>30100</v>
       </c>
       <c r="D21" s="7"/>
-    </row>
-    <row r="22" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E21" s="185"/>
+    </row>
+    <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="5" t="s">
         <v>16</v>
       </c>
@@ -3577,8 +3586,9 @@
         <v>18080</v>
       </c>
       <c r="D22" s="7"/>
-    </row>
-    <row r="23" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E22" s="185"/>
+    </row>
+    <row r="23" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="5" t="s">
         <v>17</v>
       </c>
@@ -3586,8 +3596,9 @@
         <v>6780</v>
       </c>
       <c r="D23" s="7"/>
-    </row>
-    <row r="24" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E23" s="184"/>
+    </row>
+    <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="5" t="s">
         <v>18</v>
       </c>
@@ -3595,13 +3606,17 @@
         <v>49496</v>
       </c>
       <c r="D24" s="7"/>
-    </row>
-    <row r="26" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="E24" s="184"/>
+    </row>
+    <row r="25" spans="2:5" x14ac:dyDescent="0.35">
+      <c r="E25" s="184"/>
+    </row>
+    <row r="26" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="1" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="27" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="2" t="s">
         <v>20</v>
       </c>
@@ -3609,12 +3624,12 @@
         <v>116460</v>
       </c>
     </row>
-    <row r="28" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="28" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="8" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="4" t="s">
         <v>22</v>
       </c>
@@ -3625,7 +3640,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="30" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="5" t="s">
         <v>25</v>
       </c>
@@ -3633,17 +3648,17 @@
         <v>0</v>
       </c>
       <c r="D30" s="6">
-        <v>89600</v>
-      </c>
-    </row>
-    <row r="31" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+        <v>95840</v>
+      </c>
+    </row>
+    <row r="31" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="5" t="s">
         <v>26</v>
       </c>
       <c r="C31" s="6"/>
       <c r="D31" s="6"/>
     </row>
-    <row r="32" spans="2:4" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="5" t="s">
         <v>27</v>
       </c>
@@ -57176,7 +57191,7 @@
       </c>
       <c r="M2" s="164">
         <f ca="1">COUNTIFS($D$5:$D$29,"&lt;&gt;Concluído",$F$5:$F$29,"&lt;&gt;",$F$5:$F$29,"&lt;"&amp;TODAY())</f>
-        <v>7</v>
+        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-08-18T09:04:55.714-03:00
Responsável: Júlia
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{6BA809E1-DE45-4821-8457-F19D6A798563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B67E5F4-7FF9-4050-AA8F-01A446C7F6CE}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -3118,6 +3118,27 @@
     <xf numFmtId="14" fontId="32" fillId="0" borderId="60" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="1" fontId="0" fillId="21" borderId="59" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="28" fillId="32" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="3" fontId="28" fillId="32" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3141,15 +3162,6 @@
     <xf numFmtId="0" fontId="21" fillId="9" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="29" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -3157,18 +3169,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="22" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="0" fillId="21" borderId="59" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="32" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="3" fontId="28" fillId="32" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3678,56 +3678,56 @@
   <sheetData>
     <row r="1" spans="2:7" hidden="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:7" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="170" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="171"/>
-      <c r="D2" s="171"/>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
+      <c r="B2" s="177" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="178"/>
+      <c r="D2" s="178"/>
+      <c r="E2" s="178"/>
+      <c r="F2" s="178"/>
+      <c r="G2" s="178"/>
     </row>
     <row r="3" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="172" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="173"/>
-      <c r="D3" s="173"/>
-      <c r="E3" s="173"/>
-      <c r="F3" s="173"/>
-      <c r="G3" s="174"/>
+      <c r="B3" s="179" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="180"/>
+      <c r="D3" s="180"/>
+      <c r="E3" s="180"/>
+      <c r="F3" s="180"/>
+      <c r="G3" s="181"/>
     </row>
     <row r="4" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="175"/>
-      <c r="C4" s="171"/>
-      <c r="D4" s="171"/>
-      <c r="E4" s="171"/>
-      <c r="F4" s="171"/>
-      <c r="G4" s="176"/>
+      <c r="B4" s="182"/>
+      <c r="C4" s="178"/>
+      <c r="D4" s="178"/>
+      <c r="E4" s="178"/>
+      <c r="F4" s="178"/>
+      <c r="G4" s="183"/>
     </row>
     <row r="5" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="175"/>
-      <c r="C5" s="171"/>
-      <c r="D5" s="171"/>
-      <c r="E5" s="171"/>
-      <c r="F5" s="171"/>
-      <c r="G5" s="176"/>
+      <c r="B5" s="182"/>
+      <c r="C5" s="178"/>
+      <c r="D5" s="178"/>
+      <c r="E5" s="178"/>
+      <c r="F5" s="178"/>
+      <c r="G5" s="183"/>
     </row>
     <row r="6" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="175"/>
-      <c r="C6" s="171"/>
-      <c r="D6" s="171"/>
-      <c r="E6" s="171"/>
-      <c r="F6" s="171"/>
-      <c r="G6" s="176"/>
+      <c r="B6" s="182"/>
+      <c r="C6" s="178"/>
+      <c r="D6" s="178"/>
+      <c r="E6" s="178"/>
+      <c r="F6" s="178"/>
+      <c r="G6" s="183"/>
     </row>
     <row r="7" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="177"/>
-      <c r="C7" s="178"/>
-      <c r="D7" s="178"/>
-      <c r="E7" s="178"/>
-      <c r="F7" s="178"/>
-      <c r="G7" s="179"/>
+      <c r="B7" s="184"/>
+      <c r="C7" s="185"/>
+      <c r="D7" s="185"/>
+      <c r="E7" s="185"/>
+      <c r="F7" s="185"/>
+      <c r="G7" s="186"/>
     </row>
     <row r="8" spans="2:7" hidden="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -11772,7 +11772,7 @@
       <c r="Q34" s="44"/>
     </row>
     <row r="35" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A35" s="180" t="s">
+      <c r="A35" s="187" t="s">
         <v>94</v>
       </c>
       <c r="B35" s="23">
@@ -11938,7 +11938,7 @@
       </c>
     </row>
     <row r="36" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A36" s="181"/>
+      <c r="A36" s="188"/>
       <c r="B36" s="26" t="s">
         <v>60</v>
       </c>
@@ -19203,7 +19203,7 @@
       <c r="Q80" s="44"/>
     </row>
     <row r="81" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A81" s="180" t="s">
+      <c r="A81" s="187" t="s">
         <v>137</v>
       </c>
       <c r="B81" s="23">
@@ -19369,7 +19369,7 @@
       </c>
     </row>
     <row r="82" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A82" s="182"/>
+      <c r="A82" s="189"/>
       <c r="B82" s="26" t="s">
         <v>60</v>
       </c>
@@ -20994,7 +20994,7 @@
       <c r="Q91" s="44"/>
     </row>
     <row r="92" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A92" s="180" t="s">
+      <c r="A92" s="187" t="s">
         <v>142</v>
       </c>
       <c r="B92" s="23">
@@ -21160,7 +21160,7 @@
       </c>
     </row>
     <row r="93" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A93" s="181"/>
+      <c r="A93" s="188"/>
       <c r="B93" s="26" t="s">
         <v>60</v>
       </c>
@@ -30246,25 +30246,25 @@
     <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" s="113"/>
       <c r="B1" s="114"/>
-      <c r="C1" s="183" t="s">
+      <c r="C1" s="174" t="s">
         <v>196</v>
       </c>
-      <c r="D1" s="185"/>
-      <c r="E1" s="184"/>
-      <c r="F1" s="183" t="s">
+      <c r="D1" s="176"/>
+      <c r="E1" s="175"/>
+      <c r="F1" s="174" t="s">
         <v>197</v>
       </c>
-      <c r="G1" s="185"/>
-      <c r="H1" s="184"/>
-      <c r="I1" s="183" t="s">
+      <c r="G1" s="176"/>
+      <c r="H1" s="175"/>
+      <c r="I1" s="174" t="s">
         <v>198</v>
       </c>
-      <c r="J1" s="185"/>
-      <c r="K1" s="184"/>
-      <c r="L1" s="183" t="s">
+      <c r="J1" s="176"/>
+      <c r="K1" s="175"/>
+      <c r="L1" s="174" t="s">
         <v>199</v>
       </c>
-      <c r="M1" s="184"/>
+      <c r="M1" s="175"/>
       <c r="N1" s="103"/>
       <c r="P1" s="93"/>
     </row>
@@ -56726,7 +56726,7 @@
       <c r="P1" s="10"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A2" s="190" t="s">
+      <c r="A2" s="171" t="s">
         <v>220</v>
       </c>
       <c r="B2" s="135" t="s">
@@ -56768,10 +56768,10 @@
       <c r="N2" s="167">
         <v>9469.44</v>
       </c>
-      <c r="P2" s="192"/>
+      <c r="P2" s="173"/>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A3" s="190" t="s">
+      <c r="A3" s="171" t="s">
         <v>222</v>
       </c>
       <c r="B3" s="135" t="s">
@@ -56814,12 +56814,12 @@
         <v>131214</v>
       </c>
       <c r="O3" s="10"/>
-      <c r="P3" s="191" t="s">
+      <c r="P3" s="172" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A4" s="190" t="s">
+      <c r="A4" s="171" t="s">
         <v>224</v>
       </c>
       <c r="B4" s="135" t="s">
@@ -56862,12 +56862,12 @@
         <f>M3*4</f>
         <v>888940</v>
       </c>
-      <c r="P4" s="192" t="s">
+      <c r="P4" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A5" s="190" t="s">
+      <c r="A5" s="171" t="s">
         <v>225</v>
       </c>
       <c r="B5" s="135" t="s">
@@ -56909,12 +56909,12 @@
       <c r="N5" s="167">
         <v>262428</v>
       </c>
-      <c r="P5" s="192" t="s">
+      <c r="P5" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A6" s="190" t="s">
+      <c r="A6" s="171" t="s">
         <v>226</v>
       </c>
       <c r="B6" s="135" t="s">
@@ -56956,12 +56956,12 @@
       <c r="N6" s="167">
         <v>525756</v>
       </c>
-      <c r="P6" s="192" t="s">
+      <c r="P6" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A7" s="190" t="s">
+      <c r="A7" s="171" t="s">
         <v>227</v>
       </c>
       <c r="B7" s="135" t="s">
@@ -57003,12 +57003,12 @@
       <c r="N7" s="167">
         <v>524856</v>
       </c>
-      <c r="P7" s="192" t="s">
+      <c r="P7" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A8" s="190" t="s">
+      <c r="A8" s="171" t="s">
         <v>228</v>
       </c>
       <c r="B8" s="135" t="s">
@@ -57048,12 +57048,12 @@
       <c r="N8" s="167">
         <v>818</v>
       </c>
-      <c r="P8" s="192" t="s">
+      <c r="P8" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A9" s="190" t="s">
+      <c r="A9" s="171" t="s">
         <v>229</v>
       </c>
       <c r="B9" s="135" t="s">
@@ -57095,12 +57095,12 @@
       <c r="N9" s="167">
         <v>3272</v>
       </c>
-      <c r="P9" s="192" t="s">
+      <c r="P9" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A10" s="190" t="s">
+      <c r="A10" s="171" t="s">
         <v>231</v>
       </c>
       <c r="B10" s="135" t="s">
@@ -57142,12 +57142,12 @@
       <c r="N10" s="167">
         <v>7</v>
       </c>
-      <c r="P10" s="192" t="s">
+      <c r="P10" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A11" s="190" t="s">
+      <c r="A11" s="171" t="s">
         <v>232</v>
       </c>
       <c r="B11" s="135" t="s">
@@ -57189,12 +57189,12 @@
       <c r="N11" s="167">
         <v>0</v>
       </c>
-      <c r="P11" s="192" t="s">
+      <c r="P11" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A12" s="190" t="s">
+      <c r="A12" s="171" t="s">
         <v>233</v>
       </c>
       <c r="B12" s="135" t="s">
@@ -57236,12 +57236,12 @@
       <c r="N12" s="167">
         <v>6</v>
       </c>
-      <c r="P12" s="192" t="s">
+      <c r="P12" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A13" s="190" t="s">
+      <c r="A13" s="171" t="s">
         <v>235</v>
       </c>
       <c r="B13" s="135" t="s">
@@ -57283,12 +57283,12 @@
       <c r="N13" s="167">
         <v>0</v>
       </c>
-      <c r="P13" s="192" t="s">
+      <c r="P13" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A14" s="190" t="s">
+      <c r="A14" s="171" t="s">
         <v>236</v>
       </c>
       <c r="B14" s="135" t="s">
@@ -57330,12 +57330,12 @@
       <c r="N14" s="167">
         <v>386</v>
       </c>
-      <c r="P14" s="192" t="s">
+      <c r="P14" s="173" t="s">
         <v>345</v>
       </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.35">
-      <c r="A15" s="190" t="s">
+      <c r="A15" s="171" t="s">
         <v>238</v>
       </c>
       <c r="B15" s="135" t="s">
@@ -57377,7 +57377,7 @@
       <c r="N15" s="167">
         <v>170759.97446043167</v>
       </c>
-      <c r="P15" s="191" t="s">
+      <c r="P15" s="172" t="s">
         <v>345</v>
       </c>
     </row>
@@ -57401,25 +57401,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="186" t="s">
+      <c r="A1" s="190" t="s">
         <v>240</v>
       </c>
-      <c r="B1" s="186" t="s">
+      <c r="B1" s="190" t="s">
         <v>240</v>
       </c>
-      <c r="C1" s="186" t="s">
+      <c r="C1" s="190" t="s">
         <v>240</v>
       </c>
-      <c r="D1" s="186" t="s">
+      <c r="D1" s="190" t="s">
         <v>240</v>
       </c>
-      <c r="E1" s="186" t="s">
+      <c r="E1" s="190" t="s">
         <v>240</v>
       </c>
-      <c r="F1" s="186" t="s">
+      <c r="F1" s="190" t="s">
         <v>240</v>
       </c>
-      <c r="G1" s="186" t="s">
+      <c r="G1" s="190" t="s">
         <v>240</v>
       </c>
     </row>
@@ -57754,43 +57754,43 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="30" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="187" t="s">
+      <c r="A1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="B1" s="187" t="s">
+      <c r="B1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="C1" s="187" t="s">
+      <c r="C1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="D1" s="187" t="s">
+      <c r="D1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="E1" s="187" t="s">
+      <c r="E1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="F1" s="187" t="s">
+      <c r="F1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="G1" s="187" t="s">
+      <c r="G1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="H1" s="187" t="s">
+      <c r="H1" s="191" t="s">
         <v>270</v>
       </c>
-      <c r="J1" s="188" t="s">
+      <c r="J1" s="192" t="s">
         <v>271</v>
       </c>
-      <c r="K1" s="188" t="s">
+      <c r="K1" s="192" t="s">
         <v>271</v>
       </c>
-      <c r="L1" s="188" t="s">
+      <c r="L1" s="192" t="s">
         <v>271</v>
       </c>
-      <c r="M1" s="188" t="s">
+      <c r="M1" s="192" t="s">
         <v>271</v>
       </c>
-      <c r="N1" s="188" t="s">
+      <c r="N1" s="192" t="s">
         <v>271</v>
       </c>
     </row>
@@ -57804,14 +57804,14 @@
       <c r="J2" s="149" t="s">
         <v>272</v>
       </c>
-      <c r="K2" s="189">
+      <c r="K2" s="170">
         <f>COUNTIF($D$5:$D$29,"&lt;&gt;Concluído")</f>
         <v>12</v>
       </c>
       <c r="L2" s="149" t="s">
         <v>273</v>
       </c>
-      <c r="M2" s="189">
+      <c r="M2" s="170">
         <f ca="1">COUNTIFS($D$5:$D$29,"&lt;&gt;Concluído",$F$5:$F$29,"&lt;&gt;",$F$5:$F$29,"&lt;"&amp;TODAY())</f>
         <v>11</v>
       </c>
@@ -57820,14 +57820,14 @@
       <c r="J3" s="149" t="s">
         <v>274</v>
       </c>
-      <c r="K3" s="189">
+      <c r="K3" s="170">
         <f>COUNTIF($D$5:$D$29,"Concluído")</f>
         <v>13</v>
       </c>
       <c r="L3" s="149" t="s">
         <v>275</v>
       </c>
-      <c r="M3" s="189">
+      <c r="M3" s="170">
         <f>COUNTIF($D$5:$D$29,"Impedido")</f>
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-08-18T09:20:57.772-03:00
Responsável: Júlia
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="176" documentId="13_ncr:1_{6BA809E1-DE45-4821-8457-F19D6A798563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4B67E5F4-7FF9-4050-AA8F-01A446C7F6CE}"/>
+  <xr:revisionPtr revIDLastSave="191" documentId="13_ncr:1_{6BA809E1-DE45-4821-8457-F19D6A798563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10A6EFA6-9050-4271-9700-2326DEF135C7}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -285,7 +285,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1041" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1034" uniqueCount="364">
   <si>
     <t>ACOMPANHAMENTO SUPERESTRUTURA — FOLHA DE ENTRADA</t>
   </si>
@@ -3130,15 +3130,6 @@
     <xf numFmtId="0" fontId="0" fillId="32" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3161,6 +3152,15 @@
     </xf>
     <xf numFmtId="0" fontId="21" fillId="9" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="50" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="18" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3678,56 +3678,56 @@
   <sheetData>
     <row r="1" spans="2:7" hidden="1" x14ac:dyDescent="0.35"/>
     <row r="2" spans="2:7" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B2" s="177" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" s="178"/>
-      <c r="D2" s="178"/>
-      <c r="E2" s="178"/>
-      <c r="F2" s="178"/>
-      <c r="G2" s="178"/>
+      <c r="B2" s="174" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="175"/>
+      <c r="D2" s="175"/>
+      <c r="E2" s="175"/>
+      <c r="F2" s="175"/>
+      <c r="G2" s="175"/>
     </row>
     <row r="3" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B3" s="179" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" s="180"/>
-      <c r="D3" s="180"/>
-      <c r="E3" s="180"/>
-      <c r="F3" s="180"/>
-      <c r="G3" s="181"/>
+      <c r="B3" s="176" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="177"/>
+      <c r="F3" s="177"/>
+      <c r="G3" s="178"/>
     </row>
     <row r="4" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B4" s="182"/>
-      <c r="C4" s="178"/>
-      <c r="D4" s="178"/>
-      <c r="E4" s="178"/>
-      <c r="F4" s="178"/>
-      <c r="G4" s="183"/>
+      <c r="B4" s="179"/>
+      <c r="C4" s="175"/>
+      <c r="D4" s="175"/>
+      <c r="E4" s="175"/>
+      <c r="F4" s="175"/>
+      <c r="G4" s="180"/>
     </row>
     <row r="5" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="182"/>
-      <c r="C5" s="178"/>
-      <c r="D5" s="178"/>
-      <c r="E5" s="178"/>
-      <c r="F5" s="178"/>
-      <c r="G5" s="183"/>
+      <c r="B5" s="179"/>
+      <c r="C5" s="175"/>
+      <c r="D5" s="175"/>
+      <c r="E5" s="175"/>
+      <c r="F5" s="175"/>
+      <c r="G5" s="180"/>
     </row>
     <row r="6" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="182"/>
-      <c r="C6" s="178"/>
-      <c r="D6" s="178"/>
-      <c r="E6" s="178"/>
-      <c r="F6" s="178"/>
-      <c r="G6" s="183"/>
+      <c r="B6" s="179"/>
+      <c r="C6" s="175"/>
+      <c r="D6" s="175"/>
+      <c r="E6" s="175"/>
+      <c r="F6" s="175"/>
+      <c r="G6" s="180"/>
     </row>
     <row r="7" spans="2:7" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="B7" s="184"/>
-      <c r="C7" s="185"/>
-      <c r="D7" s="185"/>
-      <c r="E7" s="185"/>
-      <c r="F7" s="185"/>
-      <c r="G7" s="186"/>
+      <c r="B7" s="181"/>
+      <c r="C7" s="182"/>
+      <c r="D7" s="182"/>
+      <c r="E7" s="182"/>
+      <c r="F7" s="182"/>
+      <c r="G7" s="183"/>
     </row>
     <row r="8" spans="2:7" hidden="1" x14ac:dyDescent="0.35"/>
     <row r="9" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -3764,63 +3764,53 @@
         <v>8</v>
       </c>
       <c r="C14" s="6">
-        <v>89400</v>
+        <v>94340</v>
       </c>
       <c r="D14" s="7">
         <f>C14</f>
-        <v>89400</v>
-      </c>
-      <c r="E14" s="150" t="s">
-        <v>345</v>
-      </c>
+        <v>94340</v>
+      </c>
+      <c r="E14" s="150"/>
     </row>
     <row r="15" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="5" t="s">
         <v>9</v>
       </c>
       <c r="C15" s="6">
-        <v>75500</v>
+        <v>79390</v>
       </c>
       <c r="D15" s="7"/>
-      <c r="E15" s="150" t="s">
-        <v>345</v>
-      </c>
+      <c r="E15" s="150"/>
     </row>
     <row r="16" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="5" t="s">
         <v>10</v>
       </c>
       <c r="C16" s="6">
-        <v>64880</v>
+        <v>71435</v>
       </c>
       <c r="D16" s="7"/>
-      <c r="E16" s="150" t="s">
-        <v>345</v>
-      </c>
+      <c r="E16" s="150"/>
     </row>
     <row r="17" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="5" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="6">
-        <v>64880</v>
+        <v>69740</v>
       </c>
       <c r="D17" s="7"/>
-      <c r="E17" s="150" t="s">
-        <v>345</v>
-      </c>
+      <c r="E17" s="150"/>
     </row>
     <row r="18" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="5" t="s">
         <v>12</v>
       </c>
       <c r="C18" s="6">
-        <v>62700</v>
+        <v>69100</v>
       </c>
       <c r="D18" s="7"/>
-      <c r="E18" s="150" t="s">
-        <v>345</v>
-      </c>
+      <c r="E18" s="150"/>
     </row>
     <row r="19" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="5" t="s">
@@ -3839,9 +3829,7 @@
         <v>44820</v>
       </c>
       <c r="D20" s="7"/>
-      <c r="E20" s="150" t="s">
-        <v>345</v>
-      </c>
+      <c r="E20" s="150"/>
     </row>
     <row r="21" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="5" t="s">
@@ -3851,9 +3839,7 @@
         <v>30600</v>
       </c>
       <c r="D21" s="7"/>
-      <c r="E21" s="150" t="s">
-        <v>345</v>
-      </c>
+      <c r="E21" s="150"/>
     </row>
     <row r="22" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="5" t="s">
@@ -3870,9 +3856,10 @@
         <v>17</v>
       </c>
       <c r="C23" s="6">
-        <v>6780</v>
+        <v>8745</v>
       </c>
       <c r="D23" s="7"/>
+      <c r="E23" s="150"/>
     </row>
     <row r="24" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="5" t="s">
@@ -11772,7 +11759,7 @@
       <c r="Q34" s="44"/>
     </row>
     <row r="35" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A35" s="187" t="s">
+      <c r="A35" s="184" t="s">
         <v>94</v>
       </c>
       <c r="B35" s="23">
@@ -11938,7 +11925,7 @@
       </c>
     </row>
     <row r="36" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A36" s="188"/>
+      <c r="A36" s="185"/>
       <c r="B36" s="26" t="s">
         <v>60</v>
       </c>
@@ -19203,7 +19190,7 @@
       <c r="Q80" s="44"/>
     </row>
     <row r="81" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A81" s="187" t="s">
+      <c r="A81" s="184" t="s">
         <v>137</v>
       </c>
       <c r="B81" s="23">
@@ -19369,7 +19356,7 @@
       </c>
     </row>
     <row r="82" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A82" s="189"/>
+      <c r="A82" s="186"/>
       <c r="B82" s="26" t="s">
         <v>60</v>
       </c>
@@ -20994,7 +20981,7 @@
       <c r="Q91" s="44"/>
     </row>
     <row r="92" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A92" s="187" t="s">
+      <c r="A92" s="184" t="s">
         <v>142</v>
       </c>
       <c r="B92" s="23">
@@ -21160,7 +21147,7 @@
       </c>
     </row>
     <row r="93" spans="1:70" x14ac:dyDescent="0.35">
-      <c r="A93" s="188"/>
+      <c r="A93" s="185"/>
       <c r="B93" s="26" t="s">
         <v>60</v>
       </c>
@@ -30246,25 +30233,25 @@
     <row r="1" spans="1:27" x14ac:dyDescent="0.35">
       <c r="A1" s="113"/>
       <c r="B1" s="114"/>
-      <c r="C1" s="174" t="s">
+      <c r="C1" s="187" t="s">
         <v>196</v>
       </c>
-      <c r="D1" s="176"/>
-      <c r="E1" s="175"/>
-      <c r="F1" s="174" t="s">
+      <c r="D1" s="189"/>
+      <c r="E1" s="188"/>
+      <c r="F1" s="187" t="s">
         <v>197</v>
       </c>
-      <c r="G1" s="176"/>
-      <c r="H1" s="175"/>
-      <c r="I1" s="174" t="s">
+      <c r="G1" s="189"/>
+      <c r="H1" s="188"/>
+      <c r="I1" s="187" t="s">
         <v>198</v>
       </c>
-      <c r="J1" s="176"/>
-      <c r="K1" s="175"/>
-      <c r="L1" s="174" t="s">
+      <c r="J1" s="189"/>
+      <c r="K1" s="188"/>
+      <c r="L1" s="187" t="s">
         <v>199</v>
       </c>
-      <c r="M1" s="175"/>
+      <c r="M1" s="188"/>
       <c r="N1" s="103"/>
       <c r="P1" s="93"/>
     </row>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-08-20T09:19:20.856-03:00
Responsável: Júlia
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/Área de Trabalho/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81044126\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="191" documentId="13_ncr:1_{6BA809E1-DE45-4821-8457-F19D6A798563}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{10A6EFA6-9050-4271-9700-2326DEF135C7}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A613191E-0F46-4A01-84CD-1391FEE8EF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27021,7 +27021,8 @@
         <v>17148</v>
       </c>
       <c r="H16" s="159">
-        <v>8090</v>
+        <f>76521-SUM(B16:G16)</f>
+        <v>10040</v>
       </c>
       <c r="I16" s="159"/>
       <c r="J16" s="159"/>
@@ -27062,7 +27063,7 @@
         <v>15</v>
       </c>
       <c r="H17" s="91">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I17" s="91"/>
       <c r="J17" s="91"/>
@@ -27109,7 +27110,7 @@
       </c>
       <c r="H18" s="91">
         <f t="shared" si="6"/>
-        <v>1011.25</v>
+        <v>1004</v>
       </c>
       <c r="I18" s="91"/>
       <c r="J18" s="91"/>
@@ -27703,7 +27704,8 @@
         <v>48321</v>
       </c>
       <c r="H27" s="159">
-        <v>22176</v>
+        <f>116759-SUM(B27:G27)</f>
+        <v>23645</v>
       </c>
       <c r="I27" s="159" t="s">
         <v>316</v>
@@ -27772,7 +27774,7 @@
         <v>18</v>
       </c>
       <c r="H28" s="91">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="I28" s="91"/>
       <c r="J28" s="91"/>
@@ -27819,7 +27821,7 @@
       </c>
       <c r="H29" s="91">
         <f t="shared" si="10"/>
-        <v>3168</v>
+        <v>2955.625</v>
       </c>
       <c r="I29" s="91"/>
       <c r="J29" s="91"/>
@@ -29123,7 +29125,8 @@
         <v>15912</v>
       </c>
       <c r="H49" s="159">
-        <v>6538</v>
+        <f>40230-SUM(B49:G49)+(900+840)/5</f>
+        <v>8728</v>
       </c>
       <c r="I49" s="159" t="s">
         <v>316</v>
@@ -29192,7 +29195,7 @@
         <v>18</v>
       </c>
       <c r="H50" s="91">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I50" s="91"/>
       <c r="J50" s="91"/>
@@ -29239,7 +29242,7 @@
       </c>
       <c r="H51" s="91">
         <f t="shared" si="18"/>
-        <v>594.36363636363637</v>
+        <v>623.42857142857144</v>
       </c>
       <c r="I51" s="91"/>
       <c r="J51" s="91"/>
@@ -29834,7 +29837,7 @@
         <v>0</v>
       </c>
       <c r="H60" s="159">
-        <v>3610</v>
+        <v>7445</v>
       </c>
       <c r="I60" s="159" t="s">
         <v>316</v>
@@ -29903,7 +29906,7 @@
         <v>0</v>
       </c>
       <c r="H61" s="91">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I61" s="91"/>
       <c r="J61" s="91"/>
@@ -29950,7 +29953,7 @@
       </c>
       <c r="H62" s="91">
         <f t="shared" si="22"/>
-        <v>1805</v>
+        <v>1861.25</v>
       </c>
       <c r="I62" s="91"/>
       <c r="J62" s="91"/>
@@ -30260,27 +30263,27 @@
       <c r="B2" s="116"/>
       <c r="C2" s="104">
         <f>SUM(C4:C733)</f>
-        <v>91764.090000000011</v>
+        <v>104517.45000000004</v>
       </c>
       <c r="D2" s="105">
         <f t="shared" ref="D2:M2" si="0">SUM(D4:D733)</f>
-        <v>89970.099999999991</v>
+        <v>102948.31999999999</v>
       </c>
       <c r="E2" s="106">
         <f t="shared" si="0"/>
-        <v>107177.90000000002</v>
+        <v>91577.900000000023</v>
       </c>
       <c r="F2" s="104">
         <f t="shared" si="0"/>
-        <v>123688.46699999996</v>
+        <v>149032.16699999999</v>
       </c>
       <c r="G2" s="105">
         <f t="shared" si="0"/>
-        <v>122280.02</v>
+        <v>147211.90000000002</v>
       </c>
       <c r="H2" s="106">
         <f t="shared" si="0"/>
-        <v>73800</v>
+        <v>50400</v>
       </c>
       <c r="I2" s="104">
         <f t="shared" si="0"/>
@@ -30292,7 +30295,7 @@
       </c>
       <c r="K2" s="106">
         <f t="shared" si="0"/>
-        <v>599999.99999999942</v>
+        <v>593684.21052631538</v>
       </c>
       <c r="L2" s="104">
         <f t="shared" si="0"/>
@@ -38883,8 +38886,12 @@
         <v>773.12</v>
       </c>
       <c r="H216" s="164"/>
-      <c r="I216" s="109"/>
-      <c r="J216" s="110"/>
+      <c r="I216" s="109">
+        <v>0</v>
+      </c>
+      <c r="J216" s="110">
+        <v>0</v>
+      </c>
       <c r="K216" s="165"/>
       <c r="L216" s="109">
         <v>0</v>
@@ -38919,8 +38926,12 @@
         <v>0</v>
       </c>
       <c r="H217" s="164"/>
-      <c r="I217" s="109"/>
-      <c r="J217" s="110"/>
+      <c r="I217" s="109">
+        <v>0</v>
+      </c>
+      <c r="J217" s="110">
+        <v>0</v>
+      </c>
       <c r="K217" s="165"/>
       <c r="L217" s="109">
         <v>0</v>
@@ -38955,8 +38966,12 @@
         <v>1380.9800000000002</v>
       </c>
       <c r="H218" s="164"/>
-      <c r="I218" s="109"/>
-      <c r="J218" s="110"/>
+      <c r="I218" s="109">
+        <v>0</v>
+      </c>
+      <c r="J218" s="110">
+        <v>0</v>
+      </c>
       <c r="K218" s="165"/>
       <c r="L218" s="109">
         <v>4631.0893098182905</v>
@@ -38977,21 +38992,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C219" s="109"/>
-      <c r="D219" s="110"/>
-      <c r="E219" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F219" s="109"/>
-      <c r="G219" s="110"/>
-      <c r="H219" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I219" s="109"/>
-      <c r="J219" s="110"/>
-      <c r="K219" s="165">
-        <v>0</v>
-      </c>
+      <c r="C219" s="109">
+        <v>121.71</v>
+      </c>
+      <c r="D219" s="110">
+        <v>1084.58</v>
+      </c>
+      <c r="E219" s="164"/>
+      <c r="F219" s="109">
+        <v>1934.99</v>
+      </c>
+      <c r="G219" s="110">
+        <v>1937.0400000000006</v>
+      </c>
+      <c r="H219" s="164"/>
+      <c r="I219" s="109">
+        <v>0</v>
+      </c>
+      <c r="J219" s="110">
+        <v>0</v>
+      </c>
+      <c r="K219" s="165"/>
       <c r="L219" s="109"/>
       <c r="M219" s="111">
         <v>4209.1000000000004</v>
@@ -39011,21 +39032,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C220" s="109"/>
-      <c r="D220" s="110"/>
-      <c r="E220" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F220" s="109"/>
-      <c r="G220" s="110"/>
-      <c r="H220" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I220" s="109"/>
-      <c r="J220" s="110"/>
-      <c r="K220" s="165">
-        <v>0</v>
-      </c>
+      <c r="C220" s="109">
+        <v>892.75</v>
+      </c>
+      <c r="D220" s="110">
+        <v>1240.0799999999997</v>
+      </c>
+      <c r="E220" s="164"/>
+      <c r="F220" s="109">
+        <v>2039.25</v>
+      </c>
+      <c r="G220" s="110">
+        <v>2198.8799999999997</v>
+      </c>
+      <c r="H220" s="164"/>
+      <c r="I220" s="109">
+        <v>0</v>
+      </c>
+      <c r="J220" s="110">
+        <v>0</v>
+      </c>
+      <c r="K220" s="165"/>
       <c r="L220" s="109"/>
       <c r="M220" s="111">
         <v>681.09999999999991</v>
@@ -39045,21 +39072,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C221" s="109"/>
-      <c r="D221" s="110"/>
-      <c r="E221" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F221" s="109"/>
-      <c r="G221" s="110"/>
-      <c r="H221" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I221" s="109"/>
-      <c r="J221" s="110"/>
-      <c r="K221" s="165">
-        <v>0</v>
-      </c>
+      <c r="C221" s="109">
+        <v>1403.8</v>
+      </c>
+      <c r="D221" s="110">
+        <v>980.1</v>
+      </c>
+      <c r="E221" s="164"/>
+      <c r="F221" s="109">
+        <v>1775.07</v>
+      </c>
+      <c r="G221" s="110">
+        <v>2018.0600000000002</v>
+      </c>
+      <c r="H221" s="164"/>
+      <c r="I221" s="109">
+        <v>0</v>
+      </c>
+      <c r="J221" s="110">
+        <v>0</v>
+      </c>
+      <c r="K221" s="165"/>
       <c r="L221" s="109"/>
       <c r="M221" s="111">
         <v>4209.1000000000004</v>
@@ -39079,21 +39112,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C222" s="109"/>
-      <c r="D222" s="110"/>
-      <c r="E222" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F222" s="109"/>
-      <c r="G222" s="110"/>
-      <c r="H222" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I222" s="109"/>
-      <c r="J222" s="110"/>
-      <c r="K222" s="165">
-        <v>0</v>
-      </c>
+      <c r="C222" s="109">
+        <v>1033.5</v>
+      </c>
+      <c r="D222" s="110">
+        <v>1171.7399999999998</v>
+      </c>
+      <c r="E222" s="164"/>
+      <c r="F222" s="109">
+        <v>1267.04</v>
+      </c>
+      <c r="G222" s="110">
+        <v>1484.7999999999997</v>
+      </c>
+      <c r="H222" s="164"/>
+      <c r="I222" s="109">
+        <v>0</v>
+      </c>
+      <c r="J222" s="110">
+        <v>0</v>
+      </c>
+      <c r="K222" s="165"/>
       <c r="L222" s="109"/>
       <c r="M222" s="111">
         <v>681.09999999999991</v>
@@ -39113,21 +39152,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C223" s="109"/>
-      <c r="D223" s="110"/>
-      <c r="E223" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F223" s="109"/>
-      <c r="G223" s="110"/>
-      <c r="H223" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I223" s="109"/>
-      <c r="J223" s="110"/>
-      <c r="K223" s="165">
-        <v>0</v>
-      </c>
+      <c r="C223" s="109">
+        <v>705.17</v>
+      </c>
+      <c r="D223" s="110">
+        <v>1481.44</v>
+      </c>
+      <c r="E223" s="164"/>
+      <c r="F223" s="109">
+        <v>373.08</v>
+      </c>
+      <c r="G223" s="110">
+        <v>1039.1399999999999</v>
+      </c>
+      <c r="H223" s="164"/>
+      <c r="I223" s="109">
+        <v>0</v>
+      </c>
+      <c r="J223" s="110">
+        <v>0</v>
+      </c>
+      <c r="K223" s="165"/>
       <c r="L223" s="109"/>
       <c r="M223" s="111">
         <v>3528</v>
@@ -39147,21 +39192,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C224" s="109"/>
-      <c r="D224" s="110"/>
-      <c r="E224" s="164">
-        <v>0</v>
-      </c>
-      <c r="F224" s="109"/>
-      <c r="G224" s="110"/>
-      <c r="H224" s="164">
-        <v>0</v>
-      </c>
-      <c r="I224" s="109"/>
-      <c r="J224" s="110"/>
-      <c r="K224" s="165">
-        <v>0</v>
-      </c>
+      <c r="C224" s="109">
+        <v>0</v>
+      </c>
+      <c r="D224" s="110">
+        <v>0</v>
+      </c>
+      <c r="E224" s="164"/>
+      <c r="F224" s="109">
+        <v>0</v>
+      </c>
+      <c r="G224" s="110">
+        <v>0</v>
+      </c>
+      <c r="H224" s="164"/>
+      <c r="I224" s="109">
+        <v>0</v>
+      </c>
+      <c r="J224" s="110">
+        <v>0</v>
+      </c>
+      <c r="K224" s="165"/>
       <c r="L224" s="109"/>
       <c r="M224" s="111">
         <v>0</v>
@@ -39181,21 +39232,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C225" s="109"/>
-      <c r="D225" s="110"/>
-      <c r="E225" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F225" s="109"/>
-      <c r="G225" s="110"/>
-      <c r="H225" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I225" s="109"/>
-      <c r="J225" s="110"/>
-      <c r="K225" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C225" s="109">
+        <v>1168.75</v>
+      </c>
+      <c r="D225" s="110">
+        <v>891.18</v>
+      </c>
+      <c r="E225" s="164"/>
+      <c r="F225" s="109">
+        <v>1288.3499999999999</v>
+      </c>
+      <c r="G225" s="110">
+        <v>1964.9199999999996</v>
+      </c>
+      <c r="H225" s="164"/>
+      <c r="I225" s="109">
+        <v>0</v>
+      </c>
+      <c r="J225" s="110">
+        <v>0</v>
+      </c>
+      <c r="K225" s="165"/>
       <c r="L225" s="109"/>
       <c r="M225" s="111">
         <v>4541.547975438596</v>
@@ -39215,21 +39272,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C226" s="109"/>
-      <c r="D226" s="110"/>
-      <c r="E226" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F226" s="109"/>
-      <c r="G226" s="110"/>
-      <c r="H226" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I226" s="109"/>
-      <c r="J226" s="110"/>
-      <c r="K226" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C226" s="109">
+        <v>1034.74</v>
+      </c>
+      <c r="D226" s="110">
+        <v>664.3599999999999</v>
+      </c>
+      <c r="E226" s="164"/>
+      <c r="F226" s="109">
+        <v>2990.92</v>
+      </c>
+      <c r="G226" s="110">
+        <v>2821.9199999999992</v>
+      </c>
+      <c r="H226" s="164"/>
+      <c r="I226" s="109">
+        <v>0</v>
+      </c>
+      <c r="J226" s="110">
+        <v>0</v>
+      </c>
+      <c r="K226" s="165"/>
       <c r="L226" s="109"/>
       <c r="M226" s="111">
         <v>4541.547975438596</v>
@@ -39249,21 +39312,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C227" s="109"/>
-      <c r="D227" s="110"/>
-      <c r="E227" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F227" s="109"/>
-      <c r="G227" s="110"/>
-      <c r="H227" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I227" s="109"/>
-      <c r="J227" s="110"/>
-      <c r="K227" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C227" s="109">
+        <v>767.13</v>
+      </c>
+      <c r="D227" s="110">
+        <v>967.90000000000009</v>
+      </c>
+      <c r="E227" s="164"/>
+      <c r="F227" s="109">
+        <v>2490.7399999999998</v>
+      </c>
+      <c r="G227" s="110">
+        <v>2626.5000000000009</v>
+      </c>
+      <c r="H227" s="164"/>
+      <c r="I227" s="109">
+        <v>0</v>
+      </c>
+      <c r="J227" s="110">
+        <v>0</v>
+      </c>
+      <c r="K227" s="165"/>
       <c r="L227" s="109"/>
       <c r="M227" s="111">
         <v>4541.547975438596</v>
@@ -39283,21 +39352,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C228" s="109"/>
-      <c r="D228" s="110"/>
-      <c r="E228" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F228" s="109"/>
-      <c r="G228" s="110"/>
-      <c r="H228" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I228" s="109"/>
-      <c r="J228" s="110"/>
-      <c r="K228" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C228" s="109">
+        <v>1326.96</v>
+      </c>
+      <c r="D228" s="110">
+        <v>879.36</v>
+      </c>
+      <c r="E228" s="164"/>
+      <c r="F228" s="109">
+        <v>2816.68</v>
+      </c>
+      <c r="G228" s="110">
+        <v>2332.8000000000006</v>
+      </c>
+      <c r="H228" s="164"/>
+      <c r="I228" s="109">
+        <v>0</v>
+      </c>
+      <c r="J228" s="110">
+        <v>0</v>
+      </c>
+      <c r="K228" s="165"/>
       <c r="L228" s="109"/>
       <c r="M228" s="111">
         <v>4541.547975438596</v>
@@ -39317,21 +39392,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C229" s="109"/>
-      <c r="D229" s="110"/>
-      <c r="E229" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F229" s="109"/>
-      <c r="G229" s="110"/>
-      <c r="H229" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I229" s="109"/>
-      <c r="J229" s="110"/>
-      <c r="K229" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C229" s="109">
+        <v>1114.3499999999999</v>
+      </c>
+      <c r="D229" s="110">
+        <v>1058.28</v>
+      </c>
+      <c r="E229" s="164"/>
+      <c r="F229" s="109">
+        <v>2242.8000000000002</v>
+      </c>
+      <c r="G229" s="110">
+        <v>2256.7199999999998</v>
+      </c>
+      <c r="H229" s="164"/>
+      <c r="I229" s="109">
+        <v>0</v>
+      </c>
+      <c r="J229" s="110">
+        <v>0</v>
+      </c>
+      <c r="K229" s="165"/>
       <c r="L229" s="109"/>
       <c r="M229" s="111">
         <v>4541.547975438596</v>
@@ -39351,21 +39432,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C230" s="109"/>
-      <c r="D230" s="110"/>
-      <c r="E230" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F230" s="109"/>
-      <c r="G230" s="110"/>
-      <c r="H230" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I230" s="109"/>
-      <c r="J230" s="110"/>
-      <c r="K230" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C230" s="109">
+        <v>340.94</v>
+      </c>
+      <c r="D230" s="110">
+        <v>656.56000000000006</v>
+      </c>
+      <c r="E230" s="164"/>
+      <c r="F230" s="109">
+        <v>1790.32</v>
+      </c>
+      <c r="G230" s="110">
+        <v>770.7600000000001</v>
+      </c>
+      <c r="H230" s="164"/>
+      <c r="I230" s="109">
+        <v>0</v>
+      </c>
+      <c r="J230" s="110">
+        <v>0</v>
+      </c>
+      <c r="K230" s="165"/>
       <c r="L230" s="109"/>
       <c r="M230" s="111">
         <v>3860.4479754385966</v>
@@ -39385,21 +39472,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C231" s="109"/>
-      <c r="D231" s="110"/>
-      <c r="E231" s="164">
-        <v>0</v>
-      </c>
-      <c r="F231" s="109"/>
-      <c r="G231" s="110"/>
-      <c r="H231" s="164">
-        <v>0</v>
-      </c>
-      <c r="I231" s="109"/>
-      <c r="J231" s="110"/>
-      <c r="K231" s="165">
-        <v>0</v>
-      </c>
+      <c r="C231" s="109">
+        <v>363.38</v>
+      </c>
+      <c r="D231" s="110">
+        <v>0</v>
+      </c>
+      <c r="E231" s="164"/>
+      <c r="F231" s="109">
+        <v>0</v>
+      </c>
+      <c r="G231" s="110">
+        <v>0</v>
+      </c>
+      <c r="H231" s="164"/>
+      <c r="I231" s="109">
+        <v>0</v>
+      </c>
+      <c r="J231" s="110">
+        <v>0</v>
+      </c>
+      <c r="K231" s="165"/>
       <c r="L231" s="109"/>
       <c r="M231" s="111">
         <v>0</v>
@@ -39419,21 +39512,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C232" s="109"/>
-      <c r="D232" s="110"/>
-      <c r="E232" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F232" s="109"/>
-      <c r="G232" s="110"/>
-      <c r="H232" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I232" s="109"/>
-      <c r="J232" s="110"/>
-      <c r="K232" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C232" s="109">
+        <v>1319.51</v>
+      </c>
+      <c r="D232" s="110">
+        <v>777.17999999999984</v>
+      </c>
+      <c r="E232" s="164"/>
+      <c r="F232" s="109">
+        <v>2243.0700000000002</v>
+      </c>
+      <c r="G232" s="110">
+        <v>1571.8400000000001</v>
+      </c>
+      <c r="H232" s="164"/>
+      <c r="I232" s="109">
+        <v>0</v>
+      </c>
+      <c r="J232" s="110">
+        <v>0</v>
+      </c>
+      <c r="K232" s="165"/>
       <c r="L232" s="109"/>
       <c r="M232" s="111">
         <v>4541.547975438596</v>
@@ -39453,21 +39552,27 @@
         <f t="shared" si="8"/>
         <v>ago/26</v>
       </c>
-      <c r="C233" s="109"/>
-      <c r="D233" s="110"/>
-      <c r="E233" s="164">
-        <v>1200</v>
-      </c>
-      <c r="F233" s="109"/>
-      <c r="G233" s="110"/>
-      <c r="H233" s="164">
-        <v>1800</v>
-      </c>
-      <c r="I233" s="109"/>
-      <c r="J233" s="110"/>
-      <c r="K233" s="165">
-        <v>789.47368421052636</v>
-      </c>
+      <c r="C233" s="109">
+        <v>1160.67</v>
+      </c>
+      <c r="D233" s="110">
+        <v>1125.4599999999998</v>
+      </c>
+      <c r="E233" s="164"/>
+      <c r="F233" s="109">
+        <v>2091.39</v>
+      </c>
+      <c r="G233" s="110">
+        <v>1908.4999999999993</v>
+      </c>
+      <c r="H233" s="164"/>
+      <c r="I233" s="109">
+        <v>0</v>
+      </c>
+      <c r="J233" s="110">
+        <v>0</v>
+      </c>
+      <c r="K233" s="165"/>
       <c r="L233" s="109"/>
       <c r="M233" s="111">
         <v>4541.547975438596</v>
@@ -57359,10 +57464,10 @@
         <v>718236.76904399996</v>
       </c>
       <c r="M15" s="167">
-        <v>176600.96402877758</v>
+        <v>180169.61151079138</v>
       </c>
       <c r="N15" s="167">
-        <v>170759.97446043167</v>
+        <v>174348.48741007198</v>
       </c>
       <c r="P15" s="172" t="s">
         <v>345</v>

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-08-20T09:20:34.649-03:00
Responsável: Júlia
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\81044126\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/Área de Trabalho/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A613191E-0F46-4A01-84CD-1391FEE8EF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{A613191E-0F46-4A01-84CD-1391FEE8EF39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{59320A00-BC07-4BAF-84C1-0F321F391647}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19090" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ENTRADA" sheetId="1" r:id="rId1"/>
@@ -3740,7 +3740,7 @@
         <v>3</v>
       </c>
       <c r="C10" s="3">
-        <v>46251</v>
+        <v>46253</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="15" customHeight="1" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
Atualiza Superestrutura · 2026-09-02T13:58:23.911-03:00
Responsável: Júlia
</commit_message>
<xml_diff>
--- a/Modelo Acompanhamento Super - FINAL.xlsx
+++ b/Modelo Acompanhamento Super - FINAL.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://globalvale-my.sharepoint.com/personal/julia_guerra_vale_com/Documents/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{069264DD-D4C4-4EFF-B52A-7C64290C7D40}"/>
+  <xr:revisionPtr revIDLastSave="40" documentId="13_ncr:1_{4854DFB7-E9B4-409C-A843-569908145318}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CAC9955B-ED76-4598-957D-FDA9243EE914}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2569,7 +2569,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="207">
+  <cellXfs count="208">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -3114,6 +3114,7 @@
     <xf numFmtId="0" fontId="24" fillId="11" borderId="0" xfId="5" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -3743,7 +3744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B1:P61"/>
+  <dimension ref="A1:P61"/>
   <sheetFormatPr defaultColWidth="8.54296875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -3753,8 +3754,8 @@
     <col min="7" max="14" width="22.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:16" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="2" spans="2:16" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="2" spans="1:16" ht="21.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="191" t="s">
         <v>0</v>
       </c>
@@ -3764,7 +3765,7 @@
       <c r="F2" s="192"/>
       <c r="G2" s="192"/>
     </row>
-    <row r="3" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="193" t="s">
         <v>1</v>
       </c>
@@ -3774,7 +3775,7 @@
       <c r="F3" s="194"/>
       <c r="G3" s="195"/>
     </row>
-    <row r="4" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="196"/>
       <c r="C4" s="192"/>
       <c r="D4" s="192"/>
@@ -3782,7 +3783,7 @@
       <c r="F4" s="192"/>
       <c r="G4" s="197"/>
     </row>
-    <row r="5" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="196"/>
       <c r="C5" s="192"/>
       <c r="D5" s="192"/>
@@ -3790,7 +3791,7 @@
       <c r="F5" s="192"/>
       <c r="G5" s="197"/>
     </row>
-    <row r="6" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="196"/>
       <c r="C6" s="192"/>
       <c r="D6" s="192"/>
@@ -3798,7 +3799,7 @@
       <c r="F6" s="192"/>
       <c r="G6" s="197"/>
     </row>
-    <row r="7" spans="2:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="198"/>
       <c r="C7" s="199"/>
       <c r="D7" s="199"/>
@@ -3806,13 +3807,13 @@
       <c r="F7" s="199"/>
       <c r="G7" s="200"/>
     </row>
-    <row r="8" spans="2:16" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="9" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="9" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="2" t="s">
         <v>3</v>
       </c>
@@ -3820,12 +3821,12 @@
         <v>46266</v>
       </c>
     </row>
-    <row r="12" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="13" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="80" t="s">
         <v>5</v>
       </c>
@@ -3868,7 +3869,8 @@
       <c r="O13" s="84"/>
       <c r="P13" s="84"/>
     </row>
-    <row r="14" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A14" s="207"/>
       <c r="B14" s="85" t="s">
         <v>6</v>
       </c>
@@ -3882,10 +3884,14 @@
         <v>97180</v>
       </c>
       <c r="F14" s="87">
-        <v>102900</v>
-      </c>
-      <c r="G14" s="86"/>
-      <c r="H14" s="87"/>
+        <v>98340</v>
+      </c>
+      <c r="G14" s="86">
+        <v>102460</v>
+      </c>
+      <c r="H14" s="87">
+        <v>104400</v>
+      </c>
       <c r="I14" s="86"/>
       <c r="J14" s="87"/>
       <c r="K14" s="86"/>
@@ -3895,7 +3901,8 @@
       <c r="O14" s="7"/>
       <c r="P14" s="7"/>
     </row>
-    <row r="15" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A15" s="207"/>
       <c r="B15" s="85" t="s">
         <v>7</v>
       </c>
@@ -3918,7 +3925,8 @@
       <c r="O15" s="7"/>
       <c r="P15" s="7"/>
     </row>
-    <row r="16" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A16" s="207"/>
       <c r="B16" s="85" t="s">
         <v>8</v>
       </c>
@@ -3941,7 +3949,8 @@
       <c r="O16" s="7"/>
       <c r="P16" s="7"/>
     </row>
-    <row r="17" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A17" s="207"/>
       <c r="B17" s="85" t="s">
         <v>9</v>
       </c>
@@ -3964,7 +3973,8 @@
       <c r="O17" s="7"/>
       <c r="P17" s="7"/>
     </row>
-    <row r="18" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A18" s="207"/>
       <c r="B18" s="85" t="s">
         <v>10</v>
       </c>
@@ -3972,20 +3982,16 @@
         <v>0</v>
       </c>
       <c r="D18" s="87">
-        <v>50260</v>
+        <v>57760</v>
       </c>
       <c r="E18" s="86">
-        <v>50540</v>
+        <v>58560</v>
       </c>
       <c r="F18" s="87">
-        <v>57660</v>
-      </c>
-      <c r="G18" s="86">
-        <v>58560</v>
-      </c>
-      <c r="H18" s="87">
-        <v>64880</v>
-      </c>
+        <v>78560</v>
+      </c>
+      <c r="G18" s="86"/>
+      <c r="H18" s="87"/>
       <c r="I18" s="86">
         <v>65400</v>
       </c>
@@ -3999,7 +4005,8 @@
       <c r="O18" s="7"/>
       <c r="P18" s="7"/>
     </row>
-    <row r="19" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A19" s="207"/>
       <c r="B19" s="85" t="s">
         <v>11</v>
       </c>
@@ -4022,7 +4029,8 @@
       <c r="O19" s="7"/>
       <c r="P19" s="7"/>
     </row>
-    <row r="20" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A20" s="207"/>
       <c r="B20" s="85" t="s">
         <v>12</v>
       </c>
@@ -4036,16 +4044,20 @@
         <v>23000</v>
       </c>
       <c r="F20" s="87">
-        <v>40120</v>
+        <v>45000</v>
       </c>
       <c r="G20" s="86">
-        <v>44820</v>
+        <v>60160</v>
       </c>
       <c r="H20" s="87">
-        <v>45000</v>
-      </c>
-      <c r="I20" s="86"/>
-      <c r="J20" s="87"/>
+        <v>64880</v>
+      </c>
+      <c r="I20" s="86">
+        <v>71775</v>
+      </c>
+      <c r="J20" s="87">
+        <v>71940</v>
+      </c>
       <c r="K20" s="86"/>
       <c r="L20" s="87"/>
       <c r="M20" s="86"/>
@@ -4053,7 +4065,8 @@
       <c r="O20" s="7"/>
       <c r="P20" s="7"/>
     </row>
-    <row r="21" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A21" s="207"/>
       <c r="B21" s="85" t="s">
         <v>13</v>
       </c>
@@ -4073,10 +4086,10 @@
         <v>35000</v>
       </c>
       <c r="H21" s="87">
-        <v>41100</v>
+        <v>39000</v>
       </c>
       <c r="I21" s="86">
-        <v>43500</v>
+        <v>40120</v>
       </c>
       <c r="J21" s="87">
         <v>44820</v>
@@ -4088,7 +4101,8 @@
       <c r="O21" s="7"/>
       <c r="P21" s="7"/>
     </row>
-    <row r="22" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A22" s="207"/>
       <c r="B22" s="85" t="s">
         <v>14</v>
       </c>
@@ -4111,7 +4125,8 @@
       <c r="O22" s="7"/>
       <c r="P22" s="7"/>
     </row>
-    <row r="23" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A23" s="207"/>
       <c r="B23" s="85" t="s">
         <v>346</v>
       </c>
@@ -4119,13 +4134,14 @@
         <v>0</v>
       </c>
       <c r="D23" s="87">
-        <v>20050</v>
+        <f>D21</f>
+        <v>21600</v>
       </c>
       <c r="E23" s="86">
         <v>23000</v>
       </c>
       <c r="F23" s="87">
-        <v>30920</v>
+        <v>31650</v>
       </c>
       <c r="G23" s="86"/>
       <c r="H23" s="87"/>
@@ -4138,7 +4154,8 @@
       <c r="O23" s="7"/>
       <c r="P23" s="7"/>
     </row>
-    <row r="24" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="207"/>
       <c r="B24" s="85" t="s">
         <v>347</v>
       </c>
@@ -4165,7 +4182,8 @@
       <c r="O24" s="7"/>
       <c r="P24" s="7"/>
     </row>
-    <row r="25" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="207"/>
       <c r="B25" s="85" t="s">
         <v>348</v>
       </c>
@@ -4204,7 +4222,8 @@
       <c r="O25" s="7"/>
       <c r="P25" s="7"/>
     </row>
-    <row r="26" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A26" s="207"/>
       <c r="B26" s="85" t="s">
         <v>349</v>
       </c>
@@ -4227,7 +4246,8 @@
       <c r="O26" s="7"/>
       <c r="P26" s="7"/>
     </row>
-    <row r="27" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A27" s="207"/>
       <c r="B27" s="85" t="s">
         <v>15</v>
       </c>
@@ -4254,12 +4274,12 @@
       <c r="O27" s="7"/>
       <c r="P27" s="7"/>
     </row>
-    <row r="29" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="1" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="30" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="2" t="s">
         <v>18</v>
       </c>
@@ -4267,12 +4287,12 @@
         <v>131260</v>
       </c>
     </row>
-    <row r="31" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="6" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="32" spans="2:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="3" t="s">
         <v>20</v>
       </c>
@@ -4291,7 +4311,8 @@
         <v>0</v>
       </c>
       <c r="D33" s="89">
-        <v>95640</v>
+        <f>D14</f>
+        <v>96100</v>
       </c>
     </row>
     <row r="34" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -4302,7 +4323,8 @@
         <v>97140</v>
       </c>
       <c r="D34" s="89">
-        <v>104980</v>
+        <f>F14</f>
+        <v>98340</v>
       </c>
     </row>
     <row r="35" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -4310,10 +4332,10 @@
         <v>25</v>
       </c>
       <c r="C35" s="89">
-        <v>110100</v>
+        <v>101220</v>
       </c>
       <c r="D35" s="89">
-        <v>110680</v>
+        <v>104500</v>
       </c>
     </row>
     <row r="36" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
@@ -4321,18 +4343,22 @@
         <v>26</v>
       </c>
       <c r="C36" s="89">
-        <v>113700</v>
+        <v>110100</v>
       </c>
       <c r="D36" s="89">
-        <v>114720</v>
+        <v>110680</v>
       </c>
     </row>
     <row r="37" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="C37" s="89"/>
-      <c r="D37" s="89"/>
+      <c r="C37" s="89">
+        <v>113700</v>
+      </c>
+      <c r="D37" s="89">
+        <v>114720</v>
+      </c>
     </row>
     <row r="38" spans="2:5" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="4" t="s">

</xml_diff>